<commit_message>
Add the needs-ticketing status
Purple fill (7030A0) on the Event Name cell means the page is live on
the website but has no tickets yet. It reads as its own status, keeping
the dashboard's colours matched to the ones the team already uses in
the spreadsheet.

These pages are published, so they count towards Live on website; the
status filter and the purple pill are what single out the three with no
tickets yet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/2026-2027 SPH Activity Master List.xlsx
+++ b/Data/2026-2027 SPH Activity Master List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Claude Working Folder\HubSpot Events - RP1 - RP4 - 2026-2027\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B67D35EE-E409-4B89-9FB5-72D978B617A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{387ABC69-274C-4A9A-BC02-40E865A4E124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38295" yWindow="0" windowWidth="38610" windowHeight="20985" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32805" yWindow="2370" windowWidth="34740" windowHeight="15345" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RP1" sheetId="1" r:id="rId1"/>
@@ -1406,7 +1406,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1443,6 +1443,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor rgb="FF33CCCC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1456,7 +1462,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1480,6 +1486,9 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4884,7 +4893,7 @@
       </c>
     </row>
     <row r="21" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="15" t="s">
         <v>250</v>
       </c>
       <c r="B21" s="7">
@@ -5390,7 +5399,7 @@
       </c>
     </row>
     <row r="29" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="15" t="s">
         <v>276</v>
       </c>
       <c r="B29" s="7">
@@ -5701,7 +5710,7 @@
       </c>
     </row>
     <row r="34" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="10" t="s">
+      <c r="A34" s="15" t="s">
         <v>286</v>
       </c>
       <c r="B34" s="7">

</xml_diff>

<commit_message>
Show "External" where a ticket count is not ours to know
Fourteen locality sessions now read "External" in the Number of Tickets
column. The build already survived that, since a non-numeric value falls
back to no count, but the word itself was discarded: the table showed a
bare dash and the detail panel hid the row, both of which read as
missing data rather than a deliberate answer.

The text is kept and shown instead, and the Ticket capacity tile says
what it covers - "across 109 of 123 sessions", with "14 booked
externally" beneath - rather than implying it totals everything.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/2026-2027 SPH Activity Master List.xlsx
+++ b/Data/2026-2027 SPH Activity Master List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Claude Working Folder\HubSpot Events - RP1 - RP4 - 2026-2027\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1BBA80-B57F-4B87-B588-795BFB7B42CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B92B8CDA-386D-4217-BF1E-E6EC7576620B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RP1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2049" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2063" uniqueCount="490">
   <si>
     <t>Event Name</t>
   </si>
@@ -1601,7 +1601,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1627,6 +1627,7 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2617,8 +2618,8 @@
       <c r="F10" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="G10" s="2">
-        <v>80</v>
+      <c r="G10" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H10" t="s">
         <v>25</v>
@@ -2812,8 +2813,8 @@
       <c r="F13" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="G13" s="2">
-        <v>80</v>
+      <c r="G13" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H13" t="s">
         <v>25</v>
@@ -3132,14 +3133,14 @@
       <c r="D18" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="13" t="s">
         <v>80</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="G18" s="2">
-        <v>80</v>
+      <c r="G18" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H18" t="s">
         <v>25</v>
@@ -4645,14 +4646,14 @@
       <c r="D11" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="13" t="s">
         <v>80</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="G11" s="2">
-        <v>80</v>
+      <c r="G11" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H11" t="s">
         <v>176</v>
@@ -6111,14 +6112,14 @@
       <c r="D34" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="E34" s="13" t="s">
         <v>80</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="G34" s="2">
-        <v>80</v>
+      <c r="G34" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H34" t="s">
         <v>176</v>
@@ -6428,14 +6429,14 @@
       <c r="D39" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="E39" s="13" t="s">
         <v>80</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="G39" s="2">
-        <v>80</v>
+      <c r="G39" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H39" t="s">
         <v>176</v>
@@ -6680,14 +6681,14 @@
       <c r="D2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="13" t="s">
         <v>80</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="G2" s="2">
-        <v>80</v>
+      <c r="G2" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H2" t="s">
         <v>320</v>
@@ -7003,14 +7004,14 @@
       <c r="D7" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="13" t="s">
         <v>80</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="G7" s="2">
-        <v>80</v>
+      <c r="G7" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H7" t="s">
         <v>320</v>
@@ -8344,14 +8345,14 @@
       <c r="D28" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="E28" s="13" t="s">
         <v>80</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="G28" s="2">
-        <v>80</v>
+      <c r="G28" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H28" t="s">
         <v>320</v>
@@ -8798,14 +8799,14 @@
       <c r="D35" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="E35" s="13" t="s">
         <v>80</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="G35" s="2">
-        <v>80</v>
+      <c r="G35" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H35" t="s">
         <v>320</v>
@@ -9099,14 +9100,14 @@
       <c r="D2" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="13" t="s">
         <v>80</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="G2" s="2">
-        <v>80</v>
+      <c r="G2" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H2" t="s">
         <v>433</v>
@@ -9809,14 +9810,14 @@
       <c r="D13" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="13" t="s">
         <v>80</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="G13" s="2">
-        <v>80</v>
+      <c r="G13" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H13" t="s">
         <v>433</v>
@@ -10062,14 +10063,14 @@
       <c r="D17" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E17" s="13" t="s">
         <v>80</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>479</v>
       </c>
-      <c r="G17" s="2">
-        <v>80</v>
+      <c r="G17" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H17" t="s">
         <v>433</v>
@@ -10190,14 +10191,14 @@
       <c r="D19" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" s="13" t="s">
         <v>80</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>483</v>
       </c>
-      <c r="G19" s="2">
-        <v>80</v>
+      <c r="G19" s="15" t="s">
+        <v>87</v>
       </c>
       <c r="H19" t="s">
         <v>433</v>

</xml_diff>